<commit_message>
feat: updated proposal skill to handle retainer phases and rounding to days/weeks estimates
</commit_message>
<xml_diff>
--- a/platforms/claude/.claude/skills/generate-proposal/assets/estimates-example.xlsx
+++ b/platforms/claude/.claude/skills/generate-proposal/assets/estimates-example.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadeemmardini/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadeemmardini/Dev/Repos/dev-agents/platforms/claude/.claude/skills/generate-proposal/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD16282-E41D-F041-870A-E42040FD7969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E209FBC-1C06-A944-8C91-391DF0469ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="254">
   <si>
     <t>Phase</t>
   </si>
@@ -795,6 +795,9 @@
   </si>
   <si>
     <t>Hour per week</t>
+  </si>
+  <si>
+    <t>Retainer Based. Monthly 5000</t>
   </si>
 </sst>
 </file>
@@ -2092,7 +2095,7 @@
       <c r="J20" s="24"/>
       <c r="K20" s="25"/>
     </row>
-    <row r="21" spans="1:11" ht="30" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="45" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -3393,7 +3396,7 @@
       <c r="J60" s="6"/>
       <c r="K60" s="12"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.2">
       <c r="A61" s="7"/>
       <c r="B61" s="7"/>
       <c r="C61" s="7" t="s">
@@ -3421,7 +3424,9 @@
         <f>I61*Variables!$B$3*Variables!$B$1</f>
         <v>6384.0000000000009</v>
       </c>
-      <c r="K61" s="13"/>
+      <c r="K61" s="13" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="9"/>
@@ -4229,12 +4234,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4376,15 +4378,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7EC52D8-A049-4D16-9A99-3EEA7A4556F5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C3DE753-9866-4886-9DE1-3A86A83C7FFD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="9dd5eb76-deb1-47dd-a327-962b84f20bd4"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4408,17 +4421,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C3DE753-9866-4886-9DE1-3A86A83C7FFD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7EC52D8-A049-4D16-9A99-3EEA7A4556F5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="9dd5eb76-deb1-47dd-a327-962b84f20bd4"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>